<commit_message>
added 2 other possible primary satellites
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanwei/Documents/MATLAB/Space EVDT 2.0/Space-EVDT/Code/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{222051E1-5E70-A648-A7FB-608B148B6815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F99A2811-39AB-5348-A497-D8EA28A67511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220"/>
+    <workbookView xWindow="4700" yWindow="-19660" windowWidth="28800" windowHeight="16220"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -404,18 +404,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
     <col min="2" max="2" width="2.7109375" customWidth="true"/>
+    <col min="4" max="4" width="4.7109375" customWidth="true"/>
+    <col min="5" max="5" width="5.7109375" customWidth="true"/>
     <col min="6" max="6" width="7.7109375" customWidth="true"/>
     <col min="7" max="9" width="2.6640625" customWidth="true"/>
     <col min="10" max="10" width="6.6640625" customWidth="true"/>
     <col min="11" max="14" width="2.6640625" customWidth="true"/>
     <col min="3" max="3" width="2.7109375" customWidth="true"/>
-    <col min="4" max="4" width="2.7109375" customWidth="true"/>
-    <col min="5" max="5" width="2.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.2">
@@ -478,7 +478,7 @@
         <v>491.49000000000001</v>
       </c>
     </row>
-    <row r="4">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.2">
       <c r="A4" s="0">
         <v>23940</v>
       </c>
@@ -496,6 +496,706 @@
       </c>
       <c r="F4" s="0">
         <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.2">
+      <c r="A5" s="0">
+        <v>47302</v>
+      </c>
+      <c r="B5" s="0">
+        <v>2</v>
+      </c>
+      <c r="C5" s="0">
+        <v>1</v>
+      </c>
+      <c r="D5" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E5" s="0">
+        <v>1</v>
+      </c>
+      <c r="F5" s="0">
+        <v>100</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.2">
+      <c r="A6" s="0">
+        <v>35934</v>
+      </c>
+      <c r="B6" s="0">
+        <v>0</v>
+      </c>
+      <c r="C6" s="0">
+        <v>0</v>
+      </c>
+      <c r="D6" s="0">
+        <v>0</v>
+      </c>
+      <c r="E6" s="0">
+        <v>0</v>
+      </c>
+      <c r="F6" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.2">
+      <c r="A7" s="0">
+        <v>28891</v>
+      </c>
+      <c r="B7" s="0">
+        <v>0</v>
+      </c>
+      <c r="C7" s="0">
+        <v>0</v>
+      </c>
+      <c r="D7" s="0">
+        <v>0</v>
+      </c>
+      <c r="E7" s="0">
+        <v>0</v>
+      </c>
+      <c r="F7" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.2">
+      <c r="A8" s="0">
+        <v>15331</v>
+      </c>
+      <c r="B8" s="0">
+        <v>0</v>
+      </c>
+      <c r="C8" s="0">
+        <v>0</v>
+      </c>
+      <c r="D8" s="0">
+        <v>0</v>
+      </c>
+      <c r="E8" s="0">
+        <v>0</v>
+      </c>
+      <c r="F8" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.2">
+      <c r="A9" s="0">
+        <v>46818</v>
+      </c>
+      <c r="B9" s="0">
+        <v>4</v>
+      </c>
+      <c r="C9" s="0">
+        <v>1</v>
+      </c>
+      <c r="D9" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E9" s="0">
+        <v>1</v>
+      </c>
+      <c r="F9" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.2">
+      <c r="A10" s="0">
+        <v>55062</v>
+      </c>
+      <c r="B10" s="0">
+        <v>4</v>
+      </c>
+      <c r="C10" s="0">
+        <v>1</v>
+      </c>
+      <c r="D10" s="0">
+        <v>1</v>
+      </c>
+      <c r="E10" s="0">
+        <v>34</v>
+      </c>
+      <c r="F10" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.2">
+      <c r="A11" s="0">
+        <v>48085</v>
+      </c>
+      <c r="B11" s="0">
+        <v>4</v>
+      </c>
+      <c r="C11" s="0">
+        <v>2</v>
+      </c>
+      <c r="D11" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="0">
+        <v>4</v>
+      </c>
+      <c r="F11" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.2">
+      <c r="A12" s="0">
+        <v>47949</v>
+      </c>
+      <c r="B12" s="0">
+        <v>4</v>
+      </c>
+      <c r="C12" s="0">
+        <v>3</v>
+      </c>
+      <c r="D12" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="0">
+        <v>1</v>
+      </c>
+      <c r="F12" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.2">
+      <c r="A13" s="0">
+        <v>46284</v>
+      </c>
+      <c r="B13" s="0">
+        <v>3</v>
+      </c>
+      <c r="C13" s="0">
+        <v>2</v>
+      </c>
+      <c r="D13" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E13" s="0">
+        <v>1</v>
+      </c>
+      <c r="F13" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.2">
+      <c r="A14" s="0">
+        <v>52713</v>
+      </c>
+      <c r="B14" s="0">
+        <v>2</v>
+      </c>
+      <c r="C14" s="0">
+        <v>1</v>
+      </c>
+      <c r="D14" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E14" s="0">
+        <v>1</v>
+      </c>
+      <c r="F14" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.2">
+      <c r="A15" s="0">
+        <v>43877</v>
+      </c>
+      <c r="B15" s="0">
+        <v>3</v>
+      </c>
+      <c r="C15" s="0">
+        <v>1</v>
+      </c>
+      <c r="D15" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E15" s="0">
+        <v>4</v>
+      </c>
+      <c r="F15" s="0">
+        <v>400</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="0">
+        <v>45049</v>
+      </c>
+      <c r="B16" s="0">
+        <v>3</v>
+      </c>
+      <c r="C16" s="0">
+        <v>3</v>
+      </c>
+      <c r="D16" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E16" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F16" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="0">
+        <v>47499</v>
+      </c>
+      <c r="B17" s="0">
+        <v>0</v>
+      </c>
+      <c r="C17" s="0">
+        <v>0</v>
+      </c>
+      <c r="D17" s="0">
+        <v>0</v>
+      </c>
+      <c r="E17" s="0">
+        <v>0</v>
+      </c>
+      <c r="F17" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.2">
+      <c r="A18" s="0">
+        <v>46455</v>
+      </c>
+      <c r="B18" s="0">
+        <v>3</v>
+      </c>
+      <c r="C18" s="0">
+        <v>1</v>
+      </c>
+      <c r="D18" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E18" s="0">
+        <v>1</v>
+      </c>
+      <c r="F18" s="0">
+        <v>42</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.2">
+      <c r="A19" s="0">
+        <v>54796</v>
+      </c>
+      <c r="B19" s="0">
+        <v>4</v>
+      </c>
+      <c r="C19" s="0">
+        <v>3</v>
+      </c>
+      <c r="D19" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E19" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F19" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.2">
+      <c r="A20" s="0">
+        <v>52758</v>
+      </c>
+      <c r="B20" s="0">
+        <v>4</v>
+      </c>
+      <c r="C20" s="0">
+        <v>1</v>
+      </c>
+      <c r="D20" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E20" s="0">
+        <v>34</v>
+      </c>
+      <c r="F20" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.2">
+      <c r="A21" s="0">
+        <v>25104</v>
+      </c>
+      <c r="B21" s="0">
+        <v>0</v>
+      </c>
+      <c r="C21" s="0">
+        <v>0</v>
+      </c>
+      <c r="D21" s="0">
+        <v>0</v>
+      </c>
+      <c r="E21" s="0">
+        <v>0</v>
+      </c>
+      <c r="F21" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.2">
+      <c r="A22" s="0">
+        <v>43180</v>
+      </c>
+      <c r="B22" s="0">
+        <v>3</v>
+      </c>
+      <c r="C22" s="0">
+        <v>1</v>
+      </c>
+      <c r="D22" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E22" s="0">
+        <v>1</v>
+      </c>
+      <c r="F22" s="0">
+        <v>100</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.2">
+      <c r="A23" s="0">
+        <v>44703</v>
+      </c>
+      <c r="B23" s="0">
+        <v>3</v>
+      </c>
+      <c r="C23" s="0">
+        <v>1</v>
+      </c>
+      <c r="D23" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E23" s="0">
+        <v>1</v>
+      </c>
+      <c r="F23" s="0">
+        <v>1500</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.2">
+      <c r="A24" s="0">
+        <v>29252</v>
+      </c>
+      <c r="B24" s="0">
+        <v>4</v>
+      </c>
+      <c r="C24" s="0">
+        <v>2</v>
+      </c>
+      <c r="D24" s="0">
+        <v>0</v>
+      </c>
+      <c r="E24" s="0">
+        <v>1</v>
+      </c>
+      <c r="F24" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>17191</v>
+      </c>
+      <c r="B25" s="0">
+        <v>0</v>
+      </c>
+      <c r="C25" s="0">
+        <v>0</v>
+      </c>
+      <c r="D25" s="0">
+        <v>0</v>
+      </c>
+      <c r="E25" s="0">
+        <v>0</v>
+      </c>
+      <c r="F25" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>18748</v>
+      </c>
+      <c r="B26" s="0">
+        <v>0</v>
+      </c>
+      <c r="C26" s="0">
+        <v>0</v>
+      </c>
+      <c r="D26" s="0">
+        <v>0</v>
+      </c>
+      <c r="E26" s="0">
+        <v>0</v>
+      </c>
+      <c r="F26" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0">
+        <v>52770</v>
+      </c>
+      <c r="B27" s="0">
+        <v>3</v>
+      </c>
+      <c r="C27" s="0">
+        <v>1</v>
+      </c>
+      <c r="D27" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E27" s="0">
+        <v>1</v>
+      </c>
+      <c r="F27" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0">
+        <v>44207</v>
+      </c>
+      <c r="B28" s="0">
+        <v>3</v>
+      </c>
+      <c r="C28" s="0">
+        <v>1</v>
+      </c>
+      <c r="D28" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E28" s="0">
+        <v>2</v>
+      </c>
+      <c r="F28" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0">
+        <v>47508</v>
+      </c>
+      <c r="B29" s="0">
+        <v>4</v>
+      </c>
+      <c r="C29" s="0">
+        <v>3</v>
+      </c>
+      <c r="D29" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E29" s="0">
+        <v>3</v>
+      </c>
+      <c r="F29" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0">
+        <v>48911</v>
+      </c>
+      <c r="B30" s="0">
+        <v>4</v>
+      </c>
+      <c r="C30" s="0">
+        <v>3</v>
+      </c>
+      <c r="D30" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E30" s="0">
+        <v>1</v>
+      </c>
+      <c r="F30" s="0">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0">
+        <v>47461</v>
+      </c>
+      <c r="B31" s="0">
+        <v>4</v>
+      </c>
+      <c r="C31" s="0">
+        <v>3</v>
+      </c>
+      <c r="D31" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E31" s="0">
+        <v>13</v>
+      </c>
+      <c r="F31" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0">
+        <v>16326</v>
+      </c>
+      <c r="B32" s="0">
+        <v>0</v>
+      </c>
+      <c r="C32" s="0">
+        <v>0</v>
+      </c>
+      <c r="D32" s="0">
+        <v>0</v>
+      </c>
+      <c r="E32" s="0">
+        <v>0</v>
+      </c>
+      <c r="F32" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0">
+        <v>47948</v>
+      </c>
+      <c r="B33" s="0">
+        <v>4</v>
+      </c>
+      <c r="C33" s="0">
+        <v>3</v>
+      </c>
+      <c r="D33" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E33" s="0">
+        <v>1</v>
+      </c>
+      <c r="F33" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0">
+        <v>20281</v>
+      </c>
+      <c r="B34" s="0">
+        <v>0</v>
+      </c>
+      <c r="C34" s="0">
+        <v>0</v>
+      </c>
+      <c r="D34" s="0">
+        <v>0</v>
+      </c>
+      <c r="E34" s="0">
+        <v>0</v>
+      </c>
+      <c r="F34" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0">
+        <v>52011</v>
+      </c>
+      <c r="B35" s="0">
+        <v>0</v>
+      </c>
+      <c r="C35" s="0">
+        <v>0</v>
+      </c>
+      <c r="D35" s="0">
+        <v>0</v>
+      </c>
+      <c r="E35" s="0">
+        <v>0</v>
+      </c>
+      <c r="F35" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0">
+        <v>47779</v>
+      </c>
+      <c r="B36" s="0">
+        <v>0</v>
+      </c>
+      <c r="C36" s="0">
+        <v>0</v>
+      </c>
+      <c r="D36" s="0">
+        <v>0</v>
+      </c>
+      <c r="E36" s="0">
+        <v>0</v>
+      </c>
+      <c r="F36" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0">
+        <v>51067</v>
+      </c>
+      <c r="B37" s="0">
+        <v>4</v>
+      </c>
+      <c r="C37" s="0">
+        <v>3</v>
+      </c>
+      <c r="D37" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E37" s="0">
+        <v>1</v>
+      </c>
+      <c r="F37" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0">
+        <v>52747</v>
+      </c>
+      <c r="B38" s="0">
+        <v>4</v>
+      </c>
+      <c r="C38" s="0">
+        <v>1</v>
+      </c>
+      <c r="D38" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E38" s="0">
+        <v>22</v>
+      </c>
+      <c r="F38" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0">
+        <v>52752</v>
+      </c>
+      <c r="B39" s="0">
+        <v>4</v>
+      </c>
+      <c r="C39" s="0">
+        <v>1</v>
+      </c>
+      <c r="D39" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E39" s="0">
+        <v>22</v>
+      </c>
+      <c r="F39" s="0">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1st attempt implementation of V model sensitivity analysis (untested)
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -404,12 +404,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
     <col min="2" max="2" width="2.7109375" customWidth="true"/>
-    <col min="4" max="4" width="4.7109375" customWidth="true"/>
+    <col min="4" max="4" width="5.7109375" customWidth="true"/>
     <col min="5" max="5" width="5.7109375" customWidth="true"/>
     <col min="6" max="6" width="7.7109375" customWidth="true"/>
     <col min="7" max="9" width="2.6640625" customWidth="true"/>
@@ -1198,6 +1198,406 @@
         <v>10</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="0">
+        <v>54844</v>
+      </c>
+      <c r="B40" s="0">
+        <v>4</v>
+      </c>
+      <c r="C40" s="0">
+        <v>3</v>
+      </c>
+      <c r="D40" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E40" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F40" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0">
+        <v>39227</v>
+      </c>
+      <c r="B41" s="0">
+        <v>3</v>
+      </c>
+      <c r="C41" s="0">
+        <v>1</v>
+      </c>
+      <c r="D41" s="0">
+        <v>0</v>
+      </c>
+      <c r="E41" s="0">
+        <v>5</v>
+      </c>
+      <c r="F41" s="0">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0">
+        <v>25994</v>
+      </c>
+      <c r="B42" s="0">
+        <v>3</v>
+      </c>
+      <c r="C42" s="0">
+        <v>1</v>
+      </c>
+      <c r="D42" s="0">
+        <v>0</v>
+      </c>
+      <c r="E42" s="0">
+        <v>1</v>
+      </c>
+      <c r="F42" s="0">
+        <v>2158</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0">
+        <v>49260</v>
+      </c>
+      <c r="B43" s="0">
+        <v>3</v>
+      </c>
+      <c r="C43" s="0">
+        <v>1</v>
+      </c>
+      <c r="D43" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E43" s="0">
+        <v>3</v>
+      </c>
+      <c r="F43" s="0">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0">
+        <v>28479</v>
+      </c>
+      <c r="B44" s="0">
+        <v>3</v>
+      </c>
+      <c r="C44" s="0">
+        <v>1</v>
+      </c>
+      <c r="D44" s="0">
+        <v>0</v>
+      </c>
+      <c r="E44" s="0">
+        <v>1</v>
+      </c>
+      <c r="F44" s="0">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0">
+        <v>27560</v>
+      </c>
+      <c r="B45" s="0">
+        <v>0</v>
+      </c>
+      <c r="C45" s="0">
+        <v>0</v>
+      </c>
+      <c r="D45" s="0">
+        <v>0</v>
+      </c>
+      <c r="E45" s="0">
+        <v>0</v>
+      </c>
+      <c r="F45" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0">
+        <v>40053</v>
+      </c>
+      <c r="B46" s="0">
+        <v>3</v>
+      </c>
+      <c r="C46" s="0">
+        <v>1</v>
+      </c>
+      <c r="D46" s="0">
+        <v>0</v>
+      </c>
+      <c r="E46" s="0">
+        <v>2</v>
+      </c>
+      <c r="F46" s="0">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0">
+        <v>41456</v>
+      </c>
+      <c r="B47" s="0">
+        <v>0</v>
+      </c>
+      <c r="C47" s="0">
+        <v>0</v>
+      </c>
+      <c r="D47" s="0">
+        <v>0</v>
+      </c>
+      <c r="E47" s="0">
+        <v>0</v>
+      </c>
+      <c r="F47" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0">
+        <v>40261</v>
+      </c>
+      <c r="B48" s="0">
+        <v>0</v>
+      </c>
+      <c r="C48" s="0">
+        <v>0</v>
+      </c>
+      <c r="D48" s="0">
+        <v>0</v>
+      </c>
+      <c r="E48" s="0">
+        <v>0</v>
+      </c>
+      <c r="F48" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0">
+        <v>43461</v>
+      </c>
+      <c r="B49" s="0">
+        <v>3</v>
+      </c>
+      <c r="C49" s="0">
+        <v>1</v>
+      </c>
+      <c r="D49" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E49" s="0">
+        <v>3</v>
+      </c>
+      <c r="F49" s="0">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0">
+        <v>39019</v>
+      </c>
+      <c r="B50" s="0">
+        <v>3</v>
+      </c>
+      <c r="C50" s="0">
+        <v>1</v>
+      </c>
+      <c r="D50" s="0">
+        <v>0</v>
+      </c>
+      <c r="E50" s="0">
+        <v>2</v>
+      </c>
+      <c r="F50" s="0">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0">
+        <v>53757</v>
+      </c>
+      <c r="B51" s="0">
+        <v>4</v>
+      </c>
+      <c r="C51" s="0">
+        <v>4</v>
+      </c>
+      <c r="D51" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E51" s="0">
+        <v>5</v>
+      </c>
+      <c r="F51" s="0">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0">
+        <v>28890</v>
+      </c>
+      <c r="B52" s="0">
+        <v>0</v>
+      </c>
+      <c r="C52" s="0">
+        <v>0</v>
+      </c>
+      <c r="D52" s="0">
+        <v>0</v>
+      </c>
+      <c r="E52" s="0">
+        <v>0</v>
+      </c>
+      <c r="F52" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0">
+        <v>40090</v>
+      </c>
+      <c r="B53" s="0">
+        <v>0</v>
+      </c>
+      <c r="C53" s="0">
+        <v>0</v>
+      </c>
+      <c r="D53" s="0">
+        <v>0</v>
+      </c>
+      <c r="E53" s="0">
+        <v>0</v>
+      </c>
+      <c r="F53" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0">
+        <v>52257</v>
+      </c>
+      <c r="B54" s="0">
+        <v>3</v>
+      </c>
+      <c r="C54" s="0">
+        <v>2</v>
+      </c>
+      <c r="D54" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="E54" s="0">
+        <v>1</v>
+      </c>
+      <c r="F54" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0">
+        <v>52983</v>
+      </c>
+      <c r="B55" s="0">
+        <v>0</v>
+      </c>
+      <c r="C55" s="0">
+        <v>0</v>
+      </c>
+      <c r="D55" s="0">
+        <v>0</v>
+      </c>
+      <c r="E55" s="0">
+        <v>0</v>
+      </c>
+      <c r="F55" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0">
+        <v>226</v>
+      </c>
+      <c r="B56" s="0">
+        <v>0</v>
+      </c>
+      <c r="C56" s="0">
+        <v>0</v>
+      </c>
+      <c r="D56" s="0">
+        <v>0</v>
+      </c>
+      <c r="E56" s="0">
+        <v>0</v>
+      </c>
+      <c r="F56" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0">
+        <v>52899</v>
+      </c>
+      <c r="B57" s="0">
+        <v>4</v>
+      </c>
+      <c r="C57" s="0">
+        <v>4</v>
+      </c>
+      <c r="D57" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E57" s="0">
+        <v>1</v>
+      </c>
+      <c r="F57" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0">
+        <v>24795</v>
+      </c>
+      <c r="B58" s="0">
+        <v>0</v>
+      </c>
+      <c r="C58" s="0">
+        <v>0</v>
+      </c>
+      <c r="D58" s="0">
+        <v>0</v>
+      </c>
+      <c r="E58" s="0">
+        <v>0</v>
+      </c>
+      <c r="F58" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0">
+        <v>52897</v>
+      </c>
+      <c r="B59" s="0">
+        <v>3</v>
+      </c>
+      <c r="C59" s="0">
+        <v>1</v>
+      </c>
+      <c r="D59" s="0">
+        <v>1</v>
+      </c>
+      <c r="E59" s="0">
+        <v>1</v>
+      </c>
+      <c r="F59" s="0">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
V model hw and socio-economic impact sensitivity analysis working
works with MC, but still debugging and data analysis to do
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
@@ -1598,6 +1598,106 @@
         <v>1</v>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="0">
+        <v>46276</v>
+      </c>
+      <c r="B60" s="0">
+        <v>3</v>
+      </c>
+      <c r="C60" s="0">
+        <v>2</v>
+      </c>
+      <c r="D60" s="0">
+        <v>0</v>
+      </c>
+      <c r="E60" s="0">
+        <v>1</v>
+      </c>
+      <c r="F60" s="0">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0">
+        <v>16881</v>
+      </c>
+      <c r="B61" s="0">
+        <v>0</v>
+      </c>
+      <c r="C61" s="0">
+        <v>0</v>
+      </c>
+      <c r="D61" s="0">
+        <v>0</v>
+      </c>
+      <c r="E61" s="0">
+        <v>0</v>
+      </c>
+      <c r="F61" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0">
+        <v>47502</v>
+      </c>
+      <c r="B62" s="0">
+        <v>3</v>
+      </c>
+      <c r="C62" s="0">
+        <v>3</v>
+      </c>
+      <c r="D62" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E62" s="0">
+        <v>24</v>
+      </c>
+      <c r="F62" s="0">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0">
+        <v>44399</v>
+      </c>
+      <c r="B63" s="0">
+        <v>3</v>
+      </c>
+      <c r="C63" s="0">
+        <v>3</v>
+      </c>
+      <c r="D63" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E63" s="0">
+        <v>1</v>
+      </c>
+      <c r="F63" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0">
+        <v>46291</v>
+      </c>
+      <c r="B64" s="0">
+        <v>0</v>
+      </c>
+      <c r="C64" s="0">
+        <v>0</v>
+      </c>
+      <c r="D64" s="0">
+        <v>0</v>
+      </c>
+      <c r="E64" s="0">
+        <v>0</v>
+      </c>
+      <c r="F64" s="0">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added isActive as Secondary_value parameter
minor improvements and corrections
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanwei/Documents/MATLAB/Space EVDT 2.0/Space-EVDT/Code/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F99A2811-39AB-5348-A497-D8EA28A67511}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB152F95-0C35-F14C-B324-717E6CD8F99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4700" yWindow="-19660" windowWidth="28800" windowHeight="16220"/>
   </bookViews>
@@ -404,18 +404,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
     <col min="2" max="2" width="2.7109375" customWidth="true"/>
     <col min="4" max="4" width="5.7109375" customWidth="true"/>
-    <col min="5" max="5" width="5.7109375" customWidth="true"/>
     <col min="6" max="6" width="7.7109375" customWidth="true"/>
-    <col min="7" max="9" width="2.6640625" customWidth="true"/>
+    <col min="7" max="7" width="2.7109375" customWidth="true"/>
     <col min="10" max="10" width="6.6640625" customWidth="true"/>
     <col min="11" max="14" width="2.6640625" customWidth="true"/>
     <col min="3" max="3" width="2.7109375" customWidth="true"/>
+    <col min="5" max="5" width="5.7109375" customWidth="true"/>
+    <col min="8" max="9" width="2.6640625" customWidth="true"/>
   </cols>
   <sheetData>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.2">
@@ -437,6 +438,9 @@
       <c r="F1" s="0">
         <v>6</v>
       </c>
+      <c r="G1" s="0">
+        <v>7</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.2">
       <c r="A2" s="0">
@@ -457,6 +461,9 @@
       <c r="F2" s="0">
         <v>0.85699999999999998</v>
       </c>
+      <c r="G2" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.2">
       <c r="A3" s="0">
@@ -477,6 +484,9 @@
       <c r="F3" s="0">
         <v>491.49000000000001</v>
       </c>
+      <c r="G3" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.2">
       <c r="A4" s="0">
@@ -497,6 +507,9 @@
       <c r="F4" s="0">
         <v>0</v>
       </c>
+      <c r="G4" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.2">
       <c r="A5" s="0">
@@ -517,6 +530,9 @@
       <c r="F5" s="0">
         <v>100</v>
       </c>
+      <c r="G5" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.2">
       <c r="A6" s="0">
@@ -537,6 +553,9 @@
       <c r="F6" s="0">
         <v>0</v>
       </c>
+      <c r="G6" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.2">
       <c r="A7" s="0">
@@ -557,6 +576,9 @@
       <c r="F7" s="0">
         <v>0</v>
       </c>
+      <c r="G7" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.2">
       <c r="A8" s="0">
@@ -577,6 +599,9 @@
       <c r="F8" s="0">
         <v>0</v>
       </c>
+      <c r="G8" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.2">
       <c r="A9" s="0">
@@ -597,6 +622,9 @@
       <c r="F9" s="0">
         <v>5</v>
       </c>
+      <c r="G9" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.2">
       <c r="A10" s="0">
@@ -617,6 +645,9 @@
       <c r="F10" s="0">
         <v>5</v>
       </c>
+      <c r="G10" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.2">
       <c r="A11" s="0">
@@ -637,6 +668,9 @@
       <c r="F11" s="0">
         <v>1</v>
       </c>
+      <c r="G11" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.2">
       <c r="A12" s="0">
@@ -657,6 +691,9 @@
       <c r="F12" s="0">
         <v>1</v>
       </c>
+      <c r="G12" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.2">
       <c r="A13" s="0">
@@ -677,6 +714,9 @@
       <c r="F13" s="0">
         <v>1</v>
       </c>
+      <c r="G13" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.2">
       <c r="A14" s="0">
@@ -697,6 +737,9 @@
       <c r="F14" s="0">
         <v>10</v>
       </c>
+      <c r="G14" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.2">
       <c r="A15" s="0">
@@ -717,6 +760,9 @@
       <c r="F15" s="0">
         <v>400</v>
       </c>
+      <c r="G15" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.2">
       <c r="A16" s="0">
@@ -737,6 +783,9 @@
       <c r="F16" s="0">
         <v>0.80000000000000004</v>
       </c>
+      <c r="G16" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.2">
       <c r="A17" s="0">
@@ -757,6 +806,9 @@
       <c r="F17" s="0">
         <v>0</v>
       </c>
+      <c r="G17" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.2">
       <c r="A18" s="0">
@@ -777,6 +829,9 @@
       <c r="F18" s="0">
         <v>42</v>
       </c>
+      <c r="G18" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.2">
       <c r="A19" s="0">
@@ -797,6 +852,9 @@
       <c r="F19" s="0">
         <v>0.80000000000000004</v>
       </c>
+      <c r="G19" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.2">
       <c r="A20" s="0">
@@ -817,6 +875,9 @@
       <c r="F20" s="0">
         <v>5</v>
       </c>
+      <c r="G20" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.2">
       <c r="A21" s="0">
@@ -837,6 +898,9 @@
       <c r="F21" s="0">
         <v>0</v>
       </c>
+      <c r="G21" s="0">
+        <v>0</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.2">
       <c r="A22" s="0">
@@ -857,6 +921,9 @@
       <c r="F22" s="0">
         <v>100</v>
       </c>
+      <c r="G22" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.2">
       <c r="A23" s="0">
@@ -877,6 +944,9 @@
       <c r="F23" s="0">
         <v>1500</v>
       </c>
+      <c r="G23" s="0">
+        <v>1</v>
+      </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.2">
       <c r="A24" s="0">
@@ -897,8 +967,11 @@
       <c r="F24" s="0">
         <v>3</v>
       </c>
-    </row>
-    <row r="25">
+      <c r="G24" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.2">
       <c r="A25" s="0">
         <v>17191</v>
       </c>
@@ -917,8 +990,11 @@
       <c r="F25" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="26">
+      <c r="G25" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.2">
       <c r="A26" s="0">
         <v>18748</v>
       </c>
@@ -937,8 +1013,11 @@
       <c r="F26" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="27">
+      <c r="G26" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.2">
       <c r="A27" s="0">
         <v>52770</v>
       </c>
@@ -957,8 +1036,11 @@
       <c r="F27" s="0">
         <v>0.80000000000000004</v>
       </c>
-    </row>
-    <row r="28">
+      <c r="G27" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.2">
       <c r="A28" s="0">
         <v>44207</v>
       </c>
@@ -977,8 +1059,11 @@
       <c r="F28" s="0">
         <v>10</v>
       </c>
-    </row>
-    <row r="29">
+      <c r="G28" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.2">
       <c r="A29" s="0">
         <v>47508</v>
       </c>
@@ -997,8 +1082,11 @@
       <c r="F29" s="0">
         <v>10</v>
       </c>
-    </row>
-    <row r="30">
+      <c r="G29" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.2">
       <c r="A30" s="0">
         <v>48911</v>
       </c>
@@ -1017,8 +1105,11 @@
       <c r="F30" s="0">
         <v>30</v>
       </c>
-    </row>
-    <row r="31">
+      <c r="G30" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" x14ac:dyDescent="0.2">
       <c r="A31" s="0">
         <v>47461</v>
       </c>
@@ -1037,8 +1128,11 @@
       <c r="F31" s="0">
         <v>5</v>
       </c>
-    </row>
-    <row r="32">
+      <c r="G31" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" x14ac:dyDescent="0.2">
       <c r="A32" s="0">
         <v>16326</v>
       </c>
@@ -1057,8 +1151,11 @@
       <c r="F32" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="33">
+      <c r="G32" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" x14ac:dyDescent="0.2">
       <c r="A33" s="0">
         <v>47948</v>
       </c>
@@ -1077,8 +1174,11 @@
       <c r="F33" s="0">
         <v>10</v>
       </c>
-    </row>
-    <row r="34">
+      <c r="G33" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.2">
       <c r="A34" s="0">
         <v>20281</v>
       </c>
@@ -1097,8 +1197,11 @@
       <c r="F34" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="35">
+      <c r="G34" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" x14ac:dyDescent="0.2">
       <c r="A35" s="0">
         <v>52011</v>
       </c>
@@ -1117,8 +1220,11 @@
       <c r="F35" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="36">
+      <c r="G35" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" x14ac:dyDescent="0.2">
       <c r="A36" s="0">
         <v>47779</v>
       </c>
@@ -1137,8 +1243,11 @@
       <c r="F36" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="37">
+      <c r="G36" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" x14ac:dyDescent="0.2">
       <c r="A37" s="0">
         <v>51067</v>
       </c>
@@ -1157,8 +1266,11 @@
       <c r="F37" s="0">
         <v>1</v>
       </c>
-    </row>
-    <row r="38">
+      <c r="G37" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" x14ac:dyDescent="0.2">
       <c r="A38" s="0">
         <v>52747</v>
       </c>
@@ -1177,8 +1289,11 @@
       <c r="F38" s="0">
         <v>10</v>
       </c>
-    </row>
-    <row r="39">
+      <c r="G38" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" x14ac:dyDescent="0.2">
       <c r="A39" s="0">
         <v>52752</v>
       </c>
@@ -1197,8 +1312,11 @@
       <c r="F39" s="0">
         <v>10</v>
       </c>
-    </row>
-    <row r="40">
+      <c r="G39" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" x14ac:dyDescent="0.2">
       <c r="A40" s="0">
         <v>54844</v>
       </c>
@@ -1217,8 +1335,11 @@
       <c r="F40" s="0">
         <v>0.80000000000000004</v>
       </c>
-    </row>
-    <row r="41">
+      <c r="G40" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" x14ac:dyDescent="0.2">
       <c r="A41" s="0">
         <v>39227</v>
       </c>
@@ -1237,8 +1358,11 @@
       <c r="F41" s="0">
         <v>250</v>
       </c>
-    </row>
-    <row r="42">
+      <c r="G41" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" x14ac:dyDescent="0.2">
       <c r="A42" s="0">
         <v>25994</v>
       </c>
@@ -1257,8 +1381,11 @@
       <c r="F42" s="0">
         <v>2158</v>
       </c>
-    </row>
-    <row r="43">
+      <c r="G42" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" x14ac:dyDescent="0.2">
       <c r="A43" s="0">
         <v>49260</v>
       </c>
@@ -1277,8 +1404,11 @@
       <c r="F43" s="0">
         <v>1000</v>
       </c>
-    </row>
-    <row r="44">
+      <c r="G43" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" x14ac:dyDescent="0.2">
       <c r="A44" s="0">
         <v>28479</v>
       </c>
@@ -1297,8 +1427,11 @@
       <c r="F44" s="0">
         <v>100</v>
       </c>
-    </row>
-    <row r="45">
+      <c r="G44" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" x14ac:dyDescent="0.2">
       <c r="A45" s="0">
         <v>27560</v>
       </c>
@@ -1317,8 +1450,11 @@
       <c r="F45" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="46">
+      <c r="G45" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" x14ac:dyDescent="0.2">
       <c r="A46" s="0">
         <v>40053</v>
       </c>
@@ -1337,8 +1473,11 @@
       <c r="F46" s="0">
         <v>498</v>
       </c>
-    </row>
-    <row r="47">
+      <c r="G46" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" x14ac:dyDescent="0.2">
       <c r="A47" s="0">
         <v>41456</v>
       </c>
@@ -1357,8 +1496,11 @@
       <c r="F47" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="48">
+      <c r="G47" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" x14ac:dyDescent="0.2">
       <c r="A48" s="0">
         <v>40261</v>
       </c>
@@ -1377,8 +1519,11 @@
       <c r="F48" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="49">
+      <c r="G48" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" x14ac:dyDescent="0.2">
       <c r="A49" s="0">
         <v>43461</v>
       </c>
@@ -1397,8 +1542,11 @@
       <c r="F49" s="0">
         <v>100</v>
       </c>
-    </row>
-    <row r="50">
+      <c r="G49" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" x14ac:dyDescent="0.2">
       <c r="A50" s="0">
         <v>39019</v>
       </c>
@@ -1417,8 +1565,11 @@
       <c r="F50" s="0">
         <v>580</v>
       </c>
-    </row>
-    <row r="51">
+      <c r="G50" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" x14ac:dyDescent="0.2">
       <c r="A51" s="0">
         <v>53757</v>
       </c>
@@ -1437,8 +1588,11 @@
       <c r="F51" s="0">
         <v>100</v>
       </c>
-    </row>
-    <row r="52">
+      <c r="G51" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" x14ac:dyDescent="0.2">
       <c r="A52" s="0">
         <v>28890</v>
       </c>
@@ -1457,8 +1611,11 @@
       <c r="F52" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="53">
+      <c r="G52" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" x14ac:dyDescent="0.2">
       <c r="A53" s="0">
         <v>40090</v>
       </c>
@@ -1477,8 +1634,11 @@
       <c r="F53" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="54">
+      <c r="G53" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" x14ac:dyDescent="0.2">
       <c r="A54" s="0">
         <v>52257</v>
       </c>
@@ -1497,8 +1657,11 @@
       <c r="F54" s="0">
         <v>50</v>
       </c>
-    </row>
-    <row r="55">
+      <c r="G54" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="55" x14ac:dyDescent="0.2">
       <c r="A55" s="0">
         <v>52983</v>
       </c>
@@ -1517,8 +1680,11 @@
       <c r="F55" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="56">
+      <c r="G55" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="56" x14ac:dyDescent="0.2">
       <c r="A56" s="0">
         <v>226</v>
       </c>
@@ -1537,8 +1703,11 @@
       <c r="F56" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="57">
+      <c r="G56" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="57" x14ac:dyDescent="0.2">
       <c r="A57" s="0">
         <v>52899</v>
       </c>
@@ -1557,8 +1726,11 @@
       <c r="F57" s="0">
         <v>1</v>
       </c>
-    </row>
-    <row r="58">
+      <c r="G57" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="58" x14ac:dyDescent="0.2">
       <c r="A58" s="0">
         <v>24795</v>
       </c>
@@ -1577,8 +1749,11 @@
       <c r="F58" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="59">
+      <c r="G58" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="59" x14ac:dyDescent="0.2">
       <c r="A59" s="0">
         <v>52897</v>
       </c>
@@ -1597,8 +1772,11 @@
       <c r="F59" s="0">
         <v>1</v>
       </c>
-    </row>
-    <row r="60">
+      <c r="G59" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="60" x14ac:dyDescent="0.2">
       <c r="A60" s="0">
         <v>46276</v>
       </c>
@@ -1617,8 +1795,11 @@
       <c r="F60" s="0">
         <v>3</v>
       </c>
-    </row>
-    <row r="61">
+      <c r="G60" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="61" x14ac:dyDescent="0.2">
       <c r="A61" s="0">
         <v>16881</v>
       </c>
@@ -1637,8 +1818,11 @@
       <c r="F61" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="62">
+      <c r="G61" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="62" x14ac:dyDescent="0.2">
       <c r="A62" s="0">
         <v>47502</v>
       </c>
@@ -1657,8 +1841,11 @@
       <c r="F62" s="0">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="63">
+      <c r="G62" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="63" x14ac:dyDescent="0.2">
       <c r="A63" s="0">
         <v>44399</v>
       </c>
@@ -1677,8 +1864,11 @@
       <c r="F63" s="0">
         <v>2</v>
       </c>
-    </row>
-    <row r="64">
+      <c r="G63" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="64" x14ac:dyDescent="0.2">
       <c r="A64" s="0">
         <v>46291</v>
       </c>
@@ -1696,6 +1886,78 @@
       </c>
       <c r="F64" s="0">
         <v>0</v>
+      </c>
+      <c r="G64" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="65" x14ac:dyDescent="0.2">
+      <c r="A65" s="0">
+        <v>39451</v>
+      </c>
+      <c r="B65" s="0">
+        <v>3</v>
+      </c>
+      <c r="C65" s="0">
+        <v>2</v>
+      </c>
+      <c r="D65" s="0">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="E65" s="0">
+        <v>3</v>
+      </c>
+      <c r="F65" s="0">
+        <v>100</v>
+      </c>
+      <c r="G65" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="66" x14ac:dyDescent="0.2">
+      <c r="A66" s="0">
+        <v>45418</v>
+      </c>
+      <c r="B66" s="0">
+        <v>0</v>
+      </c>
+      <c r="C66" s="0">
+        <v>0</v>
+      </c>
+      <c r="D66" s="0">
+        <v>0</v>
+      </c>
+      <c r="E66" s="0">
+        <v>0</v>
+      </c>
+      <c r="F66" s="0">
+        <v>0</v>
+      </c>
+      <c r="G66" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0">
+        <v>55083</v>
+      </c>
+      <c r="B67" s="0">
+        <v>4</v>
+      </c>
+      <c r="C67" s="0">
+        <v>1</v>
+      </c>
+      <c r="D67" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E67" s="0">
+        <v>36</v>
+      </c>
+      <c r="F67" s="0">
+        <v>1</v>
+      </c>
+      <c r="G67" s="0">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minor corrections, included isActive2
 included isActive2 in the selection of conjunction to analyze for V based D model
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
@@ -1960,6 +1960,328 @@
         <v>1</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="0">
+        <v>23547</v>
+      </c>
+      <c r="B68" s="0">
+        <v>0</v>
+      </c>
+      <c r="C68" s="0">
+        <v>0</v>
+      </c>
+      <c r="D68" s="0">
+        <v>0</v>
+      </c>
+      <c r="E68" s="0">
+        <v>0</v>
+      </c>
+      <c r="F68" s="0">
+        <v>0</v>
+      </c>
+      <c r="G68" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0">
+        <v>44874</v>
+      </c>
+      <c r="B69" s="0">
+        <v>3</v>
+      </c>
+      <c r="C69" s="0">
+        <v>2</v>
+      </c>
+      <c r="D69" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="E69" s="0">
+        <v>1</v>
+      </c>
+      <c r="F69" s="0">
+        <v>50</v>
+      </c>
+      <c r="G69" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0">
+        <v>41169</v>
+      </c>
+      <c r="B70" s="0">
+        <v>4</v>
+      </c>
+      <c r="C70" s="0">
+        <v>1</v>
+      </c>
+      <c r="D70" s="0">
+        <v>0</v>
+      </c>
+      <c r="E70" s="0">
+        <v>1</v>
+      </c>
+      <c r="F70" s="0">
+        <v>40</v>
+      </c>
+      <c r="G70" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0">
+        <v>54781</v>
+      </c>
+      <c r="B71" s="0">
+        <v>4</v>
+      </c>
+      <c r="C71" s="0">
+        <v>3</v>
+      </c>
+      <c r="D71" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E71" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F71" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G71" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0">
+        <v>37765</v>
+      </c>
+      <c r="B72" s="0">
+        <v>0</v>
+      </c>
+      <c r="C72" s="0">
+        <v>0</v>
+      </c>
+      <c r="D72" s="0">
+        <v>0</v>
+      </c>
+      <c r="E72" s="0">
+        <v>0</v>
+      </c>
+      <c r="F72" s="0">
+        <v>0</v>
+      </c>
+      <c r="G72" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0">
+        <v>43636</v>
+      </c>
+      <c r="B73" s="0">
+        <v>3</v>
+      </c>
+      <c r="C73" s="0">
+        <v>4</v>
+      </c>
+      <c r="D73" s="0">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="E73" s="0">
+        <v>1</v>
+      </c>
+      <c r="F73" s="0">
+        <v>10</v>
+      </c>
+      <c r="G73" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0">
+        <v>26033</v>
+      </c>
+      <c r="B74" s="0">
+        <v>0</v>
+      </c>
+      <c r="C74" s="0">
+        <v>0</v>
+      </c>
+      <c r="D74" s="0">
+        <v>0</v>
+      </c>
+      <c r="E74" s="0">
+        <v>0</v>
+      </c>
+      <c r="F74" s="0">
+        <v>0</v>
+      </c>
+      <c r="G74" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0">
+        <v>27561</v>
+      </c>
+      <c r="B75" s="0">
+        <v>0</v>
+      </c>
+      <c r="C75" s="0">
+        <v>0</v>
+      </c>
+      <c r="D75" s="0">
+        <v>0</v>
+      </c>
+      <c r="E75" s="0">
+        <v>0</v>
+      </c>
+      <c r="F75" s="0">
+        <v>0</v>
+      </c>
+      <c r="G75" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0">
+        <v>28893</v>
+      </c>
+      <c r="B76" s="0">
+        <v>0</v>
+      </c>
+      <c r="C76" s="0">
+        <v>0</v>
+      </c>
+      <c r="D76" s="0">
+        <v>0</v>
+      </c>
+      <c r="E76" s="0">
+        <v>0</v>
+      </c>
+      <c r="F76" s="0">
+        <v>0</v>
+      </c>
+      <c r="G76" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0">
+        <v>20607</v>
+      </c>
+      <c r="B77" s="0">
+        <v>0</v>
+      </c>
+      <c r="C77" s="0">
+        <v>0</v>
+      </c>
+      <c r="D77" s="0">
+        <v>0</v>
+      </c>
+      <c r="E77" s="0">
+        <v>0</v>
+      </c>
+      <c r="F77" s="0">
+        <v>0</v>
+      </c>
+      <c r="G77" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0">
+        <v>44339</v>
+      </c>
+      <c r="B78" s="0">
+        <v>3</v>
+      </c>
+      <c r="C78" s="0">
+        <v>2</v>
+      </c>
+      <c r="D78" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E78" s="0">
+        <v>1</v>
+      </c>
+      <c r="F78" s="0">
+        <v>5</v>
+      </c>
+      <c r="G78" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0">
+        <v>41770</v>
+      </c>
+      <c r="B79" s="0">
+        <v>2</v>
+      </c>
+      <c r="C79" s="0">
+        <v>1</v>
+      </c>
+      <c r="D79" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="E79" s="0">
+        <v>1</v>
+      </c>
+      <c r="F79" s="0">
+        <v>275</v>
+      </c>
+      <c r="G79" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0">
+        <v>25789</v>
+      </c>
+      <c r="B80" s="0">
+        <v>0</v>
+      </c>
+      <c r="C80" s="0">
+        <v>0</v>
+      </c>
+      <c r="D80" s="0">
+        <v>0</v>
+      </c>
+      <c r="E80" s="0">
+        <v>0</v>
+      </c>
+      <c r="F80" s="0">
+        <v>0</v>
+      </c>
+      <c r="G80" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0">
+        <v>54020</v>
+      </c>
+      <c r="B81" s="0">
+        <v>4</v>
+      </c>
+      <c r="C81" s="0">
+        <v>4</v>
+      </c>
+      <c r="D81" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="E81" s="0">
+        <v>6</v>
+      </c>
+      <c r="F81" s="0">
+        <v>12</v>
+      </c>
+      <c r="G81" s="0">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
maneuver count by conjunction not CDM
solved most bugs, only final conjunction plot bug to solve
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
@@ -2282,6 +2282,29 @@
         <v>1</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="0">
+        <v>38012</v>
+      </c>
+      <c r="B82" s="0">
+        <v>0</v>
+      </c>
+      <c r="C82" s="0">
+        <v>0</v>
+      </c>
+      <c r="D82" s="0">
+        <v>0</v>
+      </c>
+      <c r="E82" s="0">
+        <v>0</v>
+      </c>
+      <c r="F82" s="0">
+        <v>0</v>
+      </c>
+      <c r="G82" s="0">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
small corrections on sat value
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanwei/Documents/MATLAB/Space EVDT 2.0/Space-EVDT/Code/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB152F95-0C35-F14C-B324-717E6CD8F99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68CEFAD6-D500-5D4B-A767-D8F2E95427E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4700" yWindow="-19660" windowWidth="28800" windowHeight="16220"/>
   </bookViews>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
@@ -769,7 +769,7 @@
         <v>45049</v>
       </c>
       <c r="B16" s="0">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16" s="0">
         <v>3</v>
@@ -1937,7 +1937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="67" x14ac:dyDescent="0.2">
       <c r="A67" s="0">
         <v>55083</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="68" x14ac:dyDescent="0.2">
       <c r="A68" s="0">
         <v>23547</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="69" x14ac:dyDescent="0.2">
       <c r="A69" s="0">
         <v>44874</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="70" x14ac:dyDescent="0.2">
       <c r="A70" s="0">
         <v>41169</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="71" x14ac:dyDescent="0.2">
       <c r="A71" s="0">
         <v>54781</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="72" x14ac:dyDescent="0.2">
       <c r="A72" s="0">
         <v>37765</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="73" x14ac:dyDescent="0.2">
       <c r="A73" s="0">
         <v>43636</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="74" x14ac:dyDescent="0.2">
       <c r="A74" s="0">
         <v>26033</v>
       </c>
@@ -2121,7 +2121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="75" x14ac:dyDescent="0.2">
       <c r="A75" s="0">
         <v>27561</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="76" x14ac:dyDescent="0.2">
       <c r="A76" s="0">
         <v>28893</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="77" x14ac:dyDescent="0.2">
       <c r="A77" s="0">
         <v>20607</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="78" x14ac:dyDescent="0.2">
       <c r="A78" s="0">
         <v>44339</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="79" x14ac:dyDescent="0.2">
       <c r="A79" s="0">
         <v>41770</v>
       </c>
@@ -2236,7 +2236,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="80" x14ac:dyDescent="0.2">
       <c r="A80" s="0">
         <v>25789</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="81" x14ac:dyDescent="0.2">
       <c r="A81" s="0">
         <v>54020</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="82" x14ac:dyDescent="0.2">
       <c r="A82" s="0">
         <v>38012</v>
       </c>
@@ -2303,6 +2303,236 @@
       </c>
       <c r="G82" s="0">
         <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="83" x14ac:dyDescent="0.2">
+      <c r="A83" s="0">
+        <v>31119</v>
+      </c>
+      <c r="B83" s="0">
+        <v>4</v>
+      </c>
+      <c r="C83" s="0">
+        <v>3</v>
+      </c>
+      <c r="D83" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E83" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F83" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G83" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="84" x14ac:dyDescent="0.2">
+      <c r="A84" s="0">
+        <v>35933</v>
+      </c>
+      <c r="B84" s="0">
+        <v>3</v>
+      </c>
+      <c r="C84" s="0">
+        <v>2</v>
+      </c>
+      <c r="D84" s="0">
+        <v>0</v>
+      </c>
+      <c r="E84" s="0">
+        <v>1</v>
+      </c>
+      <c r="F84" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="G84" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="85" x14ac:dyDescent="0.2">
+      <c r="A85" s="0">
+        <v>48960</v>
+      </c>
+      <c r="B85" s="0">
+        <v>4</v>
+      </c>
+      <c r="C85" s="0">
+        <v>3</v>
+      </c>
+      <c r="D85" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="E85" s="0">
+        <v>20</v>
+      </c>
+      <c r="F85" s="0">
+        <v>0.78000000000000003</v>
+      </c>
+      <c r="G85" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="86" x14ac:dyDescent="0.2">
+      <c r="A86" s="0">
+        <v>24873</v>
+      </c>
+      <c r="B86" s="0">
+        <v>0</v>
+      </c>
+      <c r="C86" s="0">
+        <v>0</v>
+      </c>
+      <c r="D86" s="0">
+        <v>0</v>
+      </c>
+      <c r="E86" s="0">
+        <v>0</v>
+      </c>
+      <c r="F86" s="0">
+        <v>0</v>
+      </c>
+      <c r="G86" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="87" x14ac:dyDescent="0.2">
+      <c r="A87" s="0">
+        <v>45762</v>
+      </c>
+      <c r="B87" s="0">
+        <v>4</v>
+      </c>
+      <c r="C87" s="0">
+        <v>3</v>
+      </c>
+      <c r="D87" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="E87" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F87" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G87" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="88" x14ac:dyDescent="0.2">
+      <c r="A88" s="0">
+        <v>42825</v>
+      </c>
+      <c r="B88" s="0">
+        <v>3</v>
+      </c>
+      <c r="C88" s="0">
+        <v>1</v>
+      </c>
+      <c r="D88" s="0">
+        <v>0.75</v>
+      </c>
+      <c r="E88" s="0">
+        <v>1</v>
+      </c>
+      <c r="F88" s="0">
+        <v>150</v>
+      </c>
+      <c r="G88" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0">
+        <v>40360</v>
+      </c>
+      <c r="B89" s="0">
+        <v>3</v>
+      </c>
+      <c r="C89" s="0">
+        <v>1</v>
+      </c>
+      <c r="D89" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E89" s="0">
+        <v>1</v>
+      </c>
+      <c r="F89" s="0">
+        <v>100</v>
+      </c>
+      <c r="G89" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0">
+        <v>38755</v>
+      </c>
+      <c r="B90" s="0">
+        <v>3</v>
+      </c>
+      <c r="C90" s="0">
+        <v>1</v>
+      </c>
+      <c r="D90" s="0">
+        <v>0</v>
+      </c>
+      <c r="E90" s="0">
+        <v>1</v>
+      </c>
+      <c r="F90" s="0">
+        <v>400</v>
+      </c>
+      <c r="G90" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0">
+        <v>43943</v>
+      </c>
+      <c r="B91" s="0">
+        <v>4</v>
+      </c>
+      <c r="C91" s="0">
+        <v>1</v>
+      </c>
+      <c r="D91" s="0">
+        <v>0</v>
+      </c>
+      <c r="E91" s="0">
+        <v>130</v>
+      </c>
+      <c r="F91" s="0">
+        <v>2.8999999999999999</v>
+      </c>
+      <c r="G91" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0">
+        <v>48041</v>
+      </c>
+      <c r="B92" s="0">
+        <v>3</v>
+      </c>
+      <c r="C92" s="0">
+        <v>1</v>
+      </c>
+      <c r="D92" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E92" s="0">
+        <v>1</v>
+      </c>
+      <c r="F92" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="G92" s="0">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corrected only TLE <24h before TCA taken into account
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
@@ -2535,6 +2535,52 @@
         <v>1</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="0">
+        <v>39429</v>
+      </c>
+      <c r="B93" s="0">
+        <v>4</v>
+      </c>
+      <c r="C93" s="0">
+        <v>1</v>
+      </c>
+      <c r="D93" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E93" s="0">
+        <v>4</v>
+      </c>
+      <c r="F93" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="G93" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0">
+        <v>41901</v>
+      </c>
+      <c r="B94" s="0">
+        <v>3</v>
+      </c>
+      <c r="C94" s="0">
+        <v>1</v>
+      </c>
+      <c r="D94" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E94" s="0">
+        <v>5</v>
+      </c>
+      <c r="F94" s="0">
+        <v>5</v>
+      </c>
+      <c r="G94" s="0">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
minor changes to used database
</commit_message>
<xml_diff>
--- a/Code/Data/Secondary_value.xlsx
+++ b/Code/Data/Secondary_value.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanwei/Documents/MATLAB/Space EVDT 2.0/Space-EVDT/Code/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68CEFAD6-D500-5D4B-A767-D8F2E95427E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E83F521C-B8EA-9744-8D61-51B6591B33C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4700" yWindow="-19660" windowWidth="28800" windowHeight="16220"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029" fullCalcOnLoad="true"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B5D223-5ABE-D343-A7F1-A29E0BE91818}">
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G159"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="true"/>
@@ -447,22 +447,22 @@
         <v>35932</v>
       </c>
       <c r="B2" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C2" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2" s="0">
         <v>0</v>
       </c>
       <c r="E2" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" s="0">
-        <v>0.85699999999999998</v>
+        <v>0</v>
       </c>
       <c r="G2" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.2">
@@ -476,13 +476,13 @@
         <v>1</v>
       </c>
       <c r="D3" s="0">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E3" s="0">
         <v>2</v>
       </c>
       <c r="F3" s="0">
-        <v>491.49000000000001</v>
+        <v>511.22000000000003</v>
       </c>
       <c r="G3" s="0">
         <v>1</v>
@@ -522,13 +522,13 @@
         <v>1</v>
       </c>
       <c r="D5" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.67000000000000004</v>
       </c>
       <c r="E5" s="0">
         <v>1</v>
       </c>
       <c r="F5" s="0">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="G5" s="0">
         <v>1</v>
@@ -614,13 +614,13 @@
         <v>1</v>
       </c>
       <c r="D9" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.66000000000000003</v>
       </c>
       <c r="E9" s="0">
         <v>1</v>
       </c>
       <c r="F9" s="0">
-        <v>5</v>
+        <v>17.5</v>
       </c>
       <c r="G9" s="0">
         <v>1</v>
@@ -637,7 +637,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="0">
-        <v>1</v>
+        <v>0.88</v>
       </c>
       <c r="E10" s="0">
         <v>34</v>
@@ -654,19 +654,19 @@
         <v>48085</v>
       </c>
       <c r="B11" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C11" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D11" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E11" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F11" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="0">
         <v>1</v>
@@ -677,22 +677,22 @@
         <v>47949</v>
       </c>
       <c r="B12" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C12" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D12" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E12" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.2">
@@ -706,13 +706,13 @@
         <v>2</v>
       </c>
       <c r="D13" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.5</v>
       </c>
       <c r="E13" s="0">
         <v>1</v>
       </c>
       <c r="F13" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="0">
         <v>1</v>
@@ -729,13 +729,13 @@
         <v>1</v>
       </c>
       <c r="D14" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.88</v>
       </c>
       <c r="E14" s="0">
         <v>1</v>
       </c>
       <c r="F14" s="0">
-        <v>10</v>
+        <v>1000</v>
       </c>
       <c r="G14" s="0">
         <v>1</v>
@@ -752,13 +752,13 @@
         <v>1</v>
       </c>
       <c r="D15" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.5</v>
       </c>
       <c r="E15" s="0">
         <v>4</v>
       </c>
       <c r="F15" s="0">
-        <v>400</v>
+        <v>237</v>
       </c>
       <c r="G15" s="0">
         <v>1</v>
@@ -775,7 +775,7 @@
         <v>3</v>
       </c>
       <c r="D16" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.5</v>
       </c>
       <c r="E16" s="0">
         <v>6219</v>
@@ -821,13 +821,13 @@
         <v>1</v>
       </c>
       <c r="D18" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.64000000000000001</v>
       </c>
       <c r="E18" s="0">
         <v>1</v>
       </c>
       <c r="F18" s="0">
-        <v>42</v>
+        <v>115</v>
       </c>
       <c r="G18" s="0">
         <v>1</v>
@@ -844,7 +844,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.73999999999999999</v>
       </c>
       <c r="E19" s="0">
         <v>6219</v>
@@ -867,7 +867,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.62</v>
       </c>
       <c r="E20" s="0">
         <v>34</v>
@@ -913,13 +913,13 @@
         <v>1</v>
       </c>
       <c r="D22" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.5</v>
       </c>
       <c r="E22" s="0">
         <v>1</v>
       </c>
       <c r="F22" s="0">
-        <v>100</v>
+        <v>236.5</v>
       </c>
       <c r="G22" s="0">
         <v>1</v>
@@ -936,13 +936,13 @@
         <v>1</v>
       </c>
       <c r="D23" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.70999999999999996</v>
       </c>
       <c r="E23" s="0">
         <v>1</v>
       </c>
       <c r="F23" s="0">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="G23" s="0">
         <v>1</v>
@@ -959,13 +959,13 @@
         <v>2</v>
       </c>
       <c r="D24" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E24" s="0">
         <v>1</v>
       </c>
       <c r="F24" s="0">
-        <v>3</v>
+        <v>680</v>
       </c>
       <c r="G24" s="0">
         <v>1</v>
@@ -1022,22 +1022,22 @@
         <v>52770</v>
       </c>
       <c r="B27" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C27" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="0">
-        <v>0.80000000000000004</v>
+        <v>0</v>
       </c>
       <c r="E27" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" s="0">
-        <v>0.80000000000000004</v>
+        <v>0</v>
       </c>
       <c r="G27" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.2">
@@ -1051,7 +1051,7 @@
         <v>1</v>
       </c>
       <c r="D28" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.5</v>
       </c>
       <c r="E28" s="0">
         <v>2</v>
@@ -1074,13 +1074,13 @@
         <v>3</v>
       </c>
       <c r="D29" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.5</v>
       </c>
       <c r="E29" s="0">
         <v>3</v>
       </c>
       <c r="F29" s="0">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G29" s="0">
         <v>1</v>
@@ -1097,13 +1097,13 @@
         <v>3</v>
       </c>
       <c r="D30" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.71999999999999997</v>
       </c>
       <c r="E30" s="0">
         <v>1</v>
       </c>
       <c r="F30" s="0">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G30" s="0">
         <v>1</v>
@@ -1120,7 +1120,7 @@
         <v>3</v>
       </c>
       <c r="D31" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.5</v>
       </c>
       <c r="E31" s="0">
         <v>13</v>
@@ -1163,19 +1163,19 @@
         <v>4</v>
       </c>
       <c r="C33" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D33" s="0">
-        <v>0.80000000000000004</v>
+        <v>0</v>
       </c>
       <c r="E33" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F33" s="0">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G33" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" x14ac:dyDescent="0.2">
@@ -1258,13 +1258,13 @@
         <v>3</v>
       </c>
       <c r="D37" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.5</v>
       </c>
       <c r="E37" s="0">
         <v>1</v>
       </c>
       <c r="F37" s="0">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G37" s="0">
         <v>1</v>
@@ -1281,13 +1281,13 @@
         <v>1</v>
       </c>
       <c r="D38" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.81000000000000005</v>
       </c>
       <c r="E38" s="0">
         <v>22</v>
       </c>
       <c r="F38" s="0">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G38" s="0">
         <v>1</v>
@@ -1304,13 +1304,13 @@
         <v>1</v>
       </c>
       <c r="D39" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.81000000000000005</v>
       </c>
       <c r="E39" s="0">
         <v>22</v>
       </c>
       <c r="F39" s="0">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G39" s="0">
         <v>1</v>
@@ -1327,7 +1327,7 @@
         <v>3</v>
       </c>
       <c r="D40" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.73999999999999999</v>
       </c>
       <c r="E40" s="0">
         <v>6219</v>
@@ -1350,7 +1350,7 @@
         <v>1</v>
       </c>
       <c r="D41" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E41" s="0">
         <v>5</v>
@@ -1419,7 +1419,7 @@
         <v>1</v>
       </c>
       <c r="D44" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E44" s="0">
         <v>1</v>
@@ -1465,13 +1465,13 @@
         <v>1</v>
       </c>
       <c r="D46" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E46" s="0">
         <v>2</v>
       </c>
       <c r="F46" s="0">
-        <v>498</v>
+        <v>357</v>
       </c>
       <c r="G46" s="0">
         <v>1</v>
@@ -1534,7 +1534,7 @@
         <v>1</v>
       </c>
       <c r="D49" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.5</v>
       </c>
       <c r="E49" s="0">
         <v>3</v>
@@ -1557,13 +1557,13 @@
         <v>1</v>
       </c>
       <c r="D50" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E50" s="0">
         <v>2</v>
       </c>
       <c r="F50" s="0">
-        <v>580</v>
+        <v>507.5</v>
       </c>
       <c r="G50" s="0">
         <v>1</v>
@@ -1580,13 +1580,13 @@
         <v>4</v>
       </c>
       <c r="D51" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.84999999999999998</v>
       </c>
       <c r="E51" s="0">
         <v>5</v>
       </c>
       <c r="F51" s="0">
-        <v>100</v>
+        <v>48.5</v>
       </c>
       <c r="G51" s="0">
         <v>1</v>
@@ -1649,13 +1649,13 @@
         <v>2</v>
       </c>
       <c r="D54" s="0">
-        <v>0.75</v>
+        <v>0.80000000000000004</v>
       </c>
       <c r="E54" s="0">
         <v>1</v>
       </c>
       <c r="F54" s="0">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G54" s="0">
         <v>1</v>
@@ -1712,22 +1712,22 @@
         <v>52899</v>
       </c>
       <c r="B57" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C57" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D57" s="0">
-        <v>0.69999999999999996</v>
+        <v>0</v>
       </c>
       <c r="E57" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F57" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G57" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="58" x14ac:dyDescent="0.2">
@@ -1758,22 +1758,22 @@
         <v>52897</v>
       </c>
       <c r="B59" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C59" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D59" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E59" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F59" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="60" x14ac:dyDescent="0.2">
@@ -1787,13 +1787,13 @@
         <v>2</v>
       </c>
       <c r="D60" s="0">
-        <v>0</v>
+        <v>0.65000000000000002</v>
       </c>
       <c r="E60" s="0">
         <v>1</v>
       </c>
       <c r="F60" s="0">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="G60" s="0">
         <v>1</v>
@@ -1833,13 +1833,13 @@
         <v>3</v>
       </c>
       <c r="D62" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.68000000000000005</v>
       </c>
       <c r="E62" s="0">
         <v>24</v>
       </c>
       <c r="F62" s="0">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="G62" s="0">
         <v>1</v>
@@ -1856,13 +1856,13 @@
         <v>3</v>
       </c>
       <c r="D63" s="0">
-        <v>0.5</v>
+        <v>0.53000000000000003</v>
       </c>
       <c r="E63" s="0">
         <v>1</v>
       </c>
       <c r="F63" s="0">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G63" s="0">
         <v>1</v>
@@ -1902,13 +1902,13 @@
         <v>2</v>
       </c>
       <c r="D65" s="0">
-        <v>0.40000000000000002</v>
+        <v>0.5</v>
       </c>
       <c r="E65" s="0">
         <v>3</v>
       </c>
       <c r="F65" s="0">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G65" s="0">
         <v>1</v>
@@ -1942,22 +1942,22 @@
         <v>55083</v>
       </c>
       <c r="B67" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C67" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D67" s="0">
-        <v>0.80000000000000004</v>
+        <v>0</v>
       </c>
       <c r="E67" s="0">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="F67" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G67" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="68" x14ac:dyDescent="0.2">
@@ -1994,13 +1994,13 @@
         <v>2</v>
       </c>
       <c r="D69" s="0">
-        <v>0.29999999999999999</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="E69" s="0">
         <v>1</v>
       </c>
       <c r="F69" s="0">
-        <v>50</v>
+        <v>61.25</v>
       </c>
       <c r="G69" s="0">
         <v>1</v>
@@ -2017,13 +2017,13 @@
         <v>1</v>
       </c>
       <c r="D70" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E70" s="0">
         <v>1</v>
       </c>
       <c r="F70" s="0">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="G70" s="0">
         <v>1</v>
@@ -2040,7 +2040,7 @@
         <v>3</v>
       </c>
       <c r="D71" s="0">
-        <v>0.80000000000000004</v>
+        <v>0.73999999999999999</v>
       </c>
       <c r="E71" s="0">
         <v>6219</v>
@@ -2086,13 +2086,13 @@
         <v>4</v>
       </c>
       <c r="D73" s="0">
-        <v>0.40000000000000002</v>
+        <v>0.5</v>
       </c>
       <c r="E73" s="0">
         <v>1</v>
       </c>
       <c r="F73" s="0">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G73" s="0">
         <v>1</v>
@@ -2201,13 +2201,13 @@
         <v>2</v>
       </c>
       <c r="D78" s="0">
-        <v>0.5</v>
+        <v>0.52000000000000002</v>
       </c>
       <c r="E78" s="0">
         <v>1</v>
       </c>
       <c r="F78" s="0">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G78" s="0">
         <v>1</v>
@@ -2224,7 +2224,7 @@
         <v>1</v>
       </c>
       <c r="D79" s="0">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="E79" s="0">
         <v>1</v>
@@ -2270,7 +2270,7 @@
         <v>4</v>
       </c>
       <c r="D81" s="0">
-        <v>0.75</v>
+        <v>0.84999999999999998</v>
       </c>
       <c r="E81" s="0">
         <v>6</v>
@@ -2310,22 +2310,22 @@
         <v>31119</v>
       </c>
       <c r="B83" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C83" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D83" s="0">
-        <v>0.80000000000000004</v>
+        <v>0</v>
       </c>
       <c r="E83" s="0">
-        <v>6219</v>
+        <v>0</v>
       </c>
       <c r="F83" s="0">
-        <v>0.80000000000000004</v>
+        <v>0</v>
       </c>
       <c r="G83" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="84" x14ac:dyDescent="0.2">
@@ -2333,22 +2333,22 @@
         <v>35933</v>
       </c>
       <c r="B84" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C84" s="0">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D84" s="0">
         <v>0</v>
       </c>
       <c r="E84" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F84" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G84" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="85" x14ac:dyDescent="0.2">
@@ -2356,22 +2356,22 @@
         <v>48960</v>
       </c>
       <c r="B85" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C85" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D85" s="0">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="E85" s="0">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F85" s="0">
-        <v>0.78000000000000003</v>
+        <v>0</v>
       </c>
       <c r="G85" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="86" x14ac:dyDescent="0.2">
@@ -2408,7 +2408,7 @@
         <v>3</v>
       </c>
       <c r="D87" s="0">
-        <v>0.69999999999999996</v>
+        <v>0.5</v>
       </c>
       <c r="E87" s="0">
         <v>6219</v>
@@ -2431,7 +2431,7 @@
         <v>1</v>
       </c>
       <c r="D88" s="0">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="E88" s="0">
         <v>1</v>
@@ -2443,7 +2443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="89" x14ac:dyDescent="0.2">
       <c r="A89" s="0">
         <v>40360</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="90" x14ac:dyDescent="0.2">
       <c r="A90" s="0">
         <v>38755</v>
       </c>
@@ -2477,19 +2477,19 @@
         <v>1</v>
       </c>
       <c r="D90" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E90" s="0">
         <v>1</v>
       </c>
       <c r="F90" s="0">
-        <v>400</v>
+        <v>356</v>
       </c>
       <c r="G90" s="0">
         <v>1</v>
       </c>
     </row>
-    <row r="91">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="91" x14ac:dyDescent="0.2">
       <c r="A91" s="0">
         <v>43943</v>
       </c>
@@ -2500,65 +2500,65 @@
         <v>1</v>
       </c>
       <c r="D91" s="0">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E91" s="0">
         <v>130</v>
       </c>
       <c r="F91" s="0">
-        <v>2.8999999999999999</v>
+        <v>50</v>
       </c>
       <c r="G91" s="0">
         <v>1</v>
       </c>
     </row>
-    <row r="92">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="92" x14ac:dyDescent="0.2">
       <c r="A92" s="0">
         <v>48041</v>
       </c>
       <c r="B92" s="0">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C92" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D92" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E92" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F92" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="G92" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="93" x14ac:dyDescent="0.2">
       <c r="A93" s="0">
         <v>39429</v>
       </c>
       <c r="B93" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C93" s="0">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D93" s="0">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E93" s="0">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F93" s="0">
-        <v>0.29999999999999999</v>
+        <v>0</v>
       </c>
       <c r="G93" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="94" x14ac:dyDescent="0.2">
       <c r="A94" s="0">
         <v>41901</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>0.5</v>
       </c>
       <c r="E94" s="0">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F94" s="0">
         <v>5</v>
@@ -2581,7 +2581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="95" x14ac:dyDescent="0.2">
       <c r="A95" s="0">
         <v>54021</v>
       </c>
@@ -2592,15 +2592,1487 @@
         <v>4</v>
       </c>
       <c r="D95" s="0">
+        <v>0.84999999999999998</v>
+      </c>
+      <c r="E95" s="0">
+        <v>6</v>
+      </c>
+      <c r="F95" s="0">
+        <v>15</v>
+      </c>
+      <c r="G95" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="96" x14ac:dyDescent="0.2">
+      <c r="A96" s="0">
+        <v>26620</v>
+      </c>
+      <c r="B96" s="0">
+        <v>0</v>
+      </c>
+      <c r="C96" s="0">
+        <v>0</v>
+      </c>
+      <c r="D96" s="0">
+        <v>0</v>
+      </c>
+      <c r="E96" s="0">
+        <v>0</v>
+      </c>
+      <c r="F96" s="0">
+        <v>0</v>
+      </c>
+      <c r="G96" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="97" x14ac:dyDescent="0.2">
+      <c r="A97" s="0">
+        <v>39202</v>
+      </c>
+      <c r="B97" s="0">
+        <v>2</v>
+      </c>
+      <c r="C97" s="0">
+        <v>2</v>
+      </c>
+      <c r="D97" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E97" s="0">
+        <v>7</v>
+      </c>
+      <c r="F97" s="0">
+        <v>50</v>
+      </c>
+      <c r="G97" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="98" x14ac:dyDescent="0.2">
+      <c r="A98" s="0">
+        <v>52401</v>
+      </c>
+      <c r="B98" s="0">
+        <v>0</v>
+      </c>
+      <c r="C98" s="0">
+        <v>0</v>
+      </c>
+      <c r="D98" s="0">
+        <v>0</v>
+      </c>
+      <c r="E98" s="0">
+        <v>0</v>
+      </c>
+      <c r="F98" s="0">
+        <v>0</v>
+      </c>
+      <c r="G98" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="99" x14ac:dyDescent="0.2">
+      <c r="A99" s="0">
+        <v>45694</v>
+      </c>
+      <c r="B99" s="0">
+        <v>0</v>
+      </c>
+      <c r="C99" s="0">
+        <v>0</v>
+      </c>
+      <c r="D99" s="0">
+        <v>0</v>
+      </c>
+      <c r="E99" s="0">
+        <v>0</v>
+      </c>
+      <c r="F99" s="0">
+        <v>0</v>
+      </c>
+      <c r="G99" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="100" x14ac:dyDescent="0.2">
+      <c r="A100" s="0">
+        <v>52411</v>
+      </c>
+      <c r="B100" s="0">
+        <v>0</v>
+      </c>
+      <c r="C100" s="0">
+        <v>0</v>
+      </c>
+      <c r="D100" s="0">
+        <v>0</v>
+      </c>
+      <c r="E100" s="0">
+        <v>0</v>
+      </c>
+      <c r="F100" s="0">
+        <v>0</v>
+      </c>
+      <c r="G100" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="101" x14ac:dyDescent="0.2">
+      <c r="A101" s="0">
+        <v>47504</v>
+      </c>
+      <c r="B101" s="0">
+        <v>4</v>
+      </c>
+      <c r="C101" s="0">
+        <v>2</v>
+      </c>
+      <c r="D101" s="0">
+        <v>0.68000000000000005</v>
+      </c>
+      <c r="E101" s="0">
+        <v>1</v>
+      </c>
+      <c r="F101" s="0">
+        <v>50</v>
+      </c>
+      <c r="G101" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="102" x14ac:dyDescent="0.2">
+      <c r="A102" s="0">
+        <v>47932</v>
+      </c>
+      <c r="B102" s="0">
+        <v>3</v>
+      </c>
+      <c r="C102" s="0">
+        <v>1</v>
+      </c>
+      <c r="D102" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E102" s="0">
+        <v>1</v>
+      </c>
+      <c r="F102" s="0">
+        <v>200</v>
+      </c>
+      <c r="G102" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="103" x14ac:dyDescent="0.2">
+      <c r="A103" s="0">
+        <v>48082</v>
+      </c>
+      <c r="B103" s="0">
+        <v>0</v>
+      </c>
+      <c r="C103" s="0">
+        <v>0</v>
+      </c>
+      <c r="D103" s="0">
+        <v>0</v>
+      </c>
+      <c r="E103" s="0">
+        <v>0</v>
+      </c>
+      <c r="F103" s="0">
+        <v>0</v>
+      </c>
+      <c r="G103" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="104" x14ac:dyDescent="0.2">
+      <c r="A104" s="0">
+        <v>52766</v>
+      </c>
+      <c r="B104" s="0">
+        <v>0</v>
+      </c>
+      <c r="C104" s="0">
+        <v>0</v>
+      </c>
+      <c r="D104" s="0">
+        <v>0</v>
+      </c>
+      <c r="E104" s="0">
+        <v>0</v>
+      </c>
+      <c r="F104" s="0">
+        <v>0</v>
+      </c>
+      <c r="G104" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="105" x14ac:dyDescent="0.2">
+      <c r="A105" s="0">
+        <v>43015</v>
+      </c>
+      <c r="B105" s="0">
+        <v>0</v>
+      </c>
+      <c r="C105" s="0">
+        <v>0</v>
+      </c>
+      <c r="D105" s="0">
+        <v>0</v>
+      </c>
+      <c r="E105" s="0">
+        <v>0</v>
+      </c>
+      <c r="F105" s="0">
+        <v>0</v>
+      </c>
+      <c r="G105" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="106" x14ac:dyDescent="0.2">
+      <c r="A106" s="0">
+        <v>40380</v>
+      </c>
+      <c r="B106" s="0">
+        <v>0</v>
+      </c>
+      <c r="C106" s="0">
+        <v>0</v>
+      </c>
+      <c r="D106" s="0">
+        <v>0</v>
+      </c>
+      <c r="E106" s="0">
+        <v>0</v>
+      </c>
+      <c r="F106" s="0">
+        <v>0</v>
+      </c>
+      <c r="G106" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="107" x14ac:dyDescent="0.2">
+      <c r="A107" s="0">
+        <v>44764</v>
+      </c>
+      <c r="B107" s="0">
+        <v>4</v>
+      </c>
+      <c r="C107" s="0">
+        <v>3</v>
+      </c>
+      <c r="D107" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E107" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F107" s="0">
         <v>0.80000000000000004</v>
       </c>
-      <c r="E95" s="0">
+      <c r="G107" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="108" x14ac:dyDescent="0.2">
+      <c r="A108" s="0">
+        <v>43876</v>
+      </c>
+      <c r="B108" s="0">
+        <v>3</v>
+      </c>
+      <c r="C108" s="0">
+        <v>1</v>
+      </c>
+      <c r="D108" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E108" s="0">
+        <v>6</v>
+      </c>
+      <c r="F108" s="0">
+        <v>150</v>
+      </c>
+      <c r="G108" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="109" x14ac:dyDescent="0.2">
+      <c r="A109" s="0">
+        <v>45577</v>
+      </c>
+      <c r="B109" s="0">
+        <v>0</v>
+      </c>
+      <c r="C109" s="0">
+        <v>0</v>
+      </c>
+      <c r="D109" s="0">
+        <v>0</v>
+      </c>
+      <c r="E109" s="0">
+        <v>0</v>
+      </c>
+      <c r="F109" s="0">
+        <v>0</v>
+      </c>
+      <c r="G109" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="110" x14ac:dyDescent="0.2">
+      <c r="A110" s="0">
+        <v>44209</v>
+      </c>
+      <c r="B110" s="0">
+        <v>3</v>
+      </c>
+      <c r="C110" s="0">
+        <v>1</v>
+      </c>
+      <c r="D110" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E110" s="0">
+        <v>2</v>
+      </c>
+      <c r="F110" s="0">
+        <v>50</v>
+      </c>
+      <c r="G110" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="111" x14ac:dyDescent="0.2">
+      <c r="A111" s="0">
+        <v>48931</v>
+      </c>
+      <c r="B111" s="0">
+        <v>3</v>
+      </c>
+      <c r="C111" s="0">
+        <v>3</v>
+      </c>
+      <c r="D111" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E111" s="0">
+        <v>3</v>
+      </c>
+      <c r="F111" s="0">
+        <v>10</v>
+      </c>
+      <c r="G111" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="112" x14ac:dyDescent="0.2">
+      <c r="A112" s="0">
+        <v>48876</v>
+      </c>
+      <c r="B112" s="0">
+        <v>0</v>
+      </c>
+      <c r="C112" s="0">
+        <v>0</v>
+      </c>
+      <c r="D112" s="0">
+        <v>0</v>
+      </c>
+      <c r="E112" s="0">
+        <v>0</v>
+      </c>
+      <c r="F112" s="0">
+        <v>0</v>
+      </c>
+      <c r="G112" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="113" x14ac:dyDescent="0.2">
+      <c r="A113" s="0">
+        <v>44400</v>
+      </c>
+      <c r="B113" s="0">
+        <v>0</v>
+      </c>
+      <c r="C113" s="0">
+        <v>0</v>
+      </c>
+      <c r="D113" s="0">
+        <v>0</v>
+      </c>
+      <c r="E113" s="0">
+        <v>0</v>
+      </c>
+      <c r="F113" s="0">
+        <v>0</v>
+      </c>
+      <c r="G113" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="114" x14ac:dyDescent="0.2">
+      <c r="A114" s="0">
+        <v>40908</v>
+      </c>
+      <c r="B114" s="0">
+        <v>0</v>
+      </c>
+      <c r="C114" s="0">
+        <v>0</v>
+      </c>
+      <c r="D114" s="0">
+        <v>0</v>
+      </c>
+      <c r="E114" s="0">
+        <v>0</v>
+      </c>
+      <c r="F114" s="0">
+        <v>0</v>
+      </c>
+      <c r="G114" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="115" x14ac:dyDescent="0.2">
+      <c r="A115" s="0">
+        <v>45794</v>
+      </c>
+      <c r="B115" s="0">
+        <v>3</v>
+      </c>
+      <c r="C115" s="0">
+        <v>1</v>
+      </c>
+      <c r="D115" s="0">
+        <v>0.62</v>
+      </c>
+      <c r="E115" s="0">
         <v>5</v>
       </c>
-      <c r="F95" s="0">
+      <c r="F115" s="0">
+        <v>30</v>
+      </c>
+      <c r="G115" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="116" x14ac:dyDescent="0.2">
+      <c r="A116" s="0">
+        <v>48956</v>
+      </c>
+      <c r="B116" s="0">
+        <v>3</v>
+      </c>
+      <c r="C116" s="0">
+        <v>2</v>
+      </c>
+      <c r="D116" s="0">
+        <v>0.71999999999999997</v>
+      </c>
+      <c r="E116" s="0">
+        <v>1</v>
+      </c>
+      <c r="F116" s="0">
+        <v>5</v>
+      </c>
+      <c r="G116" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="117" x14ac:dyDescent="0.2">
+      <c r="A117" s="0">
+        <v>48902</v>
+      </c>
+      <c r="B117" s="0">
+        <v>0</v>
+      </c>
+      <c r="C117" s="0">
+        <v>0</v>
+      </c>
+      <c r="D117" s="0">
+        <v>0</v>
+      </c>
+      <c r="E117" s="0">
+        <v>0</v>
+      </c>
+      <c r="F117" s="0">
+        <v>0</v>
+      </c>
+      <c r="G117" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="118" x14ac:dyDescent="0.2">
+      <c r="A118" s="0">
+        <v>47961</v>
+      </c>
+      <c r="B118" s="0">
+        <v>0</v>
+      </c>
+      <c r="C118" s="0">
+        <v>0</v>
+      </c>
+      <c r="D118" s="0">
+        <v>0</v>
+      </c>
+      <c r="E118" s="0">
+        <v>0</v>
+      </c>
+      <c r="F118" s="0">
+        <v>0</v>
+      </c>
+      <c r="G118" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="119" x14ac:dyDescent="0.2">
+      <c r="A119" s="0">
+        <v>55077</v>
+      </c>
+      <c r="B119" s="0">
+        <v>0</v>
+      </c>
+      <c r="C119" s="0">
+        <v>0</v>
+      </c>
+      <c r="D119" s="0">
+        <v>0</v>
+      </c>
+      <c r="E119" s="0">
+        <v>0</v>
+      </c>
+      <c r="F119" s="0">
+        <v>0</v>
+      </c>
+      <c r="G119" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="120" x14ac:dyDescent="0.2">
+      <c r="A120" s="0">
+        <v>54807</v>
+      </c>
+      <c r="B120" s="0">
+        <v>4</v>
+      </c>
+      <c r="C120" s="0">
+        <v>3</v>
+      </c>
+      <c r="D120" s="0">
+        <v>0.73999999999999999</v>
+      </c>
+      <c r="E120" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F120" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G120" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="121" x14ac:dyDescent="0.2">
+      <c r="A121" s="0">
+        <v>45779</v>
+      </c>
+      <c r="B121" s="0">
+        <v>4</v>
+      </c>
+      <c r="C121" s="0">
+        <v>3</v>
+      </c>
+      <c r="D121" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E121" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F121" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G121" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="122" x14ac:dyDescent="0.2">
+      <c r="A122" s="0">
+        <v>55067</v>
+      </c>
+      <c r="B122" s="0">
+        <v>0</v>
+      </c>
+      <c r="C122" s="0">
+        <v>0</v>
+      </c>
+      <c r="D122" s="0">
+        <v>0</v>
+      </c>
+      <c r="E122" s="0">
+        <v>0</v>
+      </c>
+      <c r="F122" s="0">
+        <v>0</v>
+      </c>
+      <c r="G122" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="123" x14ac:dyDescent="0.2">
+      <c r="A123" s="0">
+        <v>55064</v>
+      </c>
+      <c r="B123" s="0">
+        <v>3</v>
+      </c>
+      <c r="C123" s="0">
+        <v>1</v>
+      </c>
+      <c r="D123" s="0">
+        <v>0.73999999999999999</v>
+      </c>
+      <c r="E123" s="0">
+        <v>28</v>
+      </c>
+      <c r="F123" s="0">
+        <v>10</v>
+      </c>
+      <c r="G123" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="0">
+        <v>52023</v>
+      </c>
+      <c r="B124" s="0">
+        <v>0</v>
+      </c>
+      <c r="C124" s="0">
+        <v>0</v>
+      </c>
+      <c r="D124" s="0">
+        <v>0</v>
+      </c>
+      <c r="E124" s="0">
+        <v>0</v>
+      </c>
+      <c r="F124" s="0">
+        <v>0</v>
+      </c>
+      <c r="G124" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="0">
+        <v>51058</v>
+      </c>
+      <c r="B125" s="0">
+        <v>0</v>
+      </c>
+      <c r="C125" s="0">
+        <v>0</v>
+      </c>
+      <c r="D125" s="0">
+        <v>0</v>
+      </c>
+      <c r="E125" s="0">
+        <v>0</v>
+      </c>
+      <c r="F125" s="0">
+        <v>0</v>
+      </c>
+      <c r="G125" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="0">
+        <v>52767</v>
+      </c>
+      <c r="B126" s="0">
+        <v>0</v>
+      </c>
+      <c r="C126" s="0">
+        <v>0</v>
+      </c>
+      <c r="D126" s="0">
+        <v>0</v>
+      </c>
+      <c r="E126" s="0">
+        <v>0</v>
+      </c>
+      <c r="F126" s="0">
+        <v>0</v>
+      </c>
+      <c r="G126" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="0">
+        <v>48951</v>
+      </c>
+      <c r="B127" s="0">
+        <v>4</v>
+      </c>
+      <c r="C127" s="0">
+        <v>2</v>
+      </c>
+      <c r="D127" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E127" s="0">
+        <v>1</v>
+      </c>
+      <c r="F127" s="0">
         <v>8</v>
       </c>
-      <c r="G95" s="0">
+      <c r="G127" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="0">
+        <v>51471</v>
+      </c>
+      <c r="B128" s="0">
+        <v>4</v>
+      </c>
+      <c r="C128" s="0">
+        <v>3</v>
+      </c>
+      <c r="D128" s="0">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="E128" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F128" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G128" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="0">
+        <v>26365</v>
+      </c>
+      <c r="B129" s="0">
+        <v>0</v>
+      </c>
+      <c r="C129" s="0">
+        <v>0</v>
+      </c>
+      <c r="D129" s="0">
+        <v>0</v>
+      </c>
+      <c r="E129" s="0">
+        <v>0</v>
+      </c>
+      <c r="F129" s="0">
+        <v>0</v>
+      </c>
+      <c r="G129" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="0">
+        <v>55066</v>
+      </c>
+      <c r="B130" s="0">
+        <v>0</v>
+      </c>
+      <c r="C130" s="0">
+        <v>0</v>
+      </c>
+      <c r="D130" s="0">
+        <v>0</v>
+      </c>
+      <c r="E130" s="0">
+        <v>0</v>
+      </c>
+      <c r="F130" s="0">
+        <v>0</v>
+      </c>
+      <c r="G130" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="0">
+        <v>55028</v>
+      </c>
+      <c r="B131" s="0">
+        <v>0</v>
+      </c>
+      <c r="C131" s="0">
+        <v>0</v>
+      </c>
+      <c r="D131" s="0">
+        <v>0</v>
+      </c>
+      <c r="E131" s="0">
+        <v>0</v>
+      </c>
+      <c r="F131" s="0">
+        <v>0</v>
+      </c>
+      <c r="G131" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="0">
+        <v>49071</v>
+      </c>
+      <c r="B132" s="0">
+        <v>3</v>
+      </c>
+      <c r="C132" s="0">
+        <v>1</v>
+      </c>
+      <c r="D132" s="0">
+        <v>0.73999999999999999</v>
+      </c>
+      <c r="E132" s="0">
+        <v>2</v>
+      </c>
+      <c r="F132" s="0">
+        <v>25</v>
+      </c>
+      <c r="G132" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="0">
+        <v>41890</v>
+      </c>
+      <c r="B133" s="0">
+        <v>3</v>
+      </c>
+      <c r="C133" s="0">
+        <v>2</v>
+      </c>
+      <c r="D133" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E133" s="0">
+        <v>8</v>
+      </c>
+      <c r="F133" s="0">
+        <v>10</v>
+      </c>
+      <c r="G133" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="0">
+        <v>55050</v>
+      </c>
+      <c r="B134" s="0">
+        <v>3</v>
+      </c>
+      <c r="C134" s="0">
+        <v>1</v>
+      </c>
+      <c r="D134" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E134" s="0">
+        <v>24</v>
+      </c>
+      <c r="F134" s="0">
+        <v>25</v>
+      </c>
+      <c r="G134" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="0">
+        <v>46281</v>
+      </c>
+      <c r="B135" s="0">
+        <v>0</v>
+      </c>
+      <c r="C135" s="0">
+        <v>0</v>
+      </c>
+      <c r="D135" s="0">
+        <v>0</v>
+      </c>
+      <c r="E135" s="0">
+        <v>0</v>
+      </c>
+      <c r="F135" s="0">
+        <v>0</v>
+      </c>
+      <c r="G135" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="0">
+        <v>51036</v>
+      </c>
+      <c r="B136" s="0">
+        <v>0</v>
+      </c>
+      <c r="C136" s="0">
+        <v>0</v>
+      </c>
+      <c r="D136" s="0">
+        <v>0</v>
+      </c>
+      <c r="E136" s="0">
+        <v>0</v>
+      </c>
+      <c r="F136" s="0">
+        <v>0</v>
+      </c>
+      <c r="G136" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="0">
+        <v>52417</v>
+      </c>
+      <c r="B137" s="0">
+        <v>0</v>
+      </c>
+      <c r="C137" s="0">
+        <v>0</v>
+      </c>
+      <c r="D137" s="0">
+        <v>0</v>
+      </c>
+      <c r="E137" s="0">
+        <v>0</v>
+      </c>
+      <c r="F137" s="0">
+        <v>0</v>
+      </c>
+      <c r="G137" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="0">
+        <v>51008</v>
+      </c>
+      <c r="B138" s="0">
+        <v>4</v>
+      </c>
+      <c r="C138" s="0">
+        <v>1</v>
+      </c>
+      <c r="D138" s="0">
+        <v>0.78000000000000003</v>
+      </c>
+      <c r="E138" s="0">
+        <v>34</v>
+      </c>
+      <c r="F138" s="0">
+        <v>5</v>
+      </c>
+      <c r="G138" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="0">
+        <v>41908</v>
+      </c>
+      <c r="B139" s="0">
+        <v>3</v>
+      </c>
+      <c r="C139" s="0">
+        <v>1</v>
+      </c>
+      <c r="D139" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="E139" s="0">
+        <v>4</v>
+      </c>
+      <c r="F139" s="0">
+        <v>100</v>
+      </c>
+      <c r="G139" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="0">
+        <v>55101</v>
+      </c>
+      <c r="B140" s="0">
+        <v>0</v>
+      </c>
+      <c r="C140" s="0">
+        <v>0</v>
+      </c>
+      <c r="D140" s="0">
+        <v>0</v>
+      </c>
+      <c r="E140" s="0">
+        <v>0</v>
+      </c>
+      <c r="F140" s="0">
+        <v>0</v>
+      </c>
+      <c r="G140" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="0">
+        <v>51657</v>
+      </c>
+      <c r="B141" s="0">
+        <v>0</v>
+      </c>
+      <c r="C141" s="0">
+        <v>0</v>
+      </c>
+      <c r="D141" s="0">
+        <v>0</v>
+      </c>
+      <c r="E141" s="0">
+        <v>0</v>
+      </c>
+      <c r="F141" s="0">
+        <v>0</v>
+      </c>
+      <c r="G141" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="0">
+        <v>47892</v>
+      </c>
+      <c r="B142" s="0">
+        <v>4</v>
+      </c>
+      <c r="C142" s="0">
+        <v>3</v>
+      </c>
+      <c r="D142" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E142" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F142" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G142" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="0">
+        <v>46296</v>
+      </c>
+      <c r="B143" s="0">
+        <v>0</v>
+      </c>
+      <c r="C143" s="0">
+        <v>0</v>
+      </c>
+      <c r="D143" s="0">
+        <v>0</v>
+      </c>
+      <c r="E143" s="0">
+        <v>0</v>
+      </c>
+      <c r="F143" s="0">
+        <v>0</v>
+      </c>
+      <c r="G143" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="0">
+        <v>55035</v>
+      </c>
+      <c r="B144" s="0">
+        <v>0</v>
+      </c>
+      <c r="C144" s="0">
+        <v>0</v>
+      </c>
+      <c r="D144" s="0">
+        <v>0</v>
+      </c>
+      <c r="E144" s="0">
+        <v>0</v>
+      </c>
+      <c r="F144" s="0">
+        <v>0</v>
+      </c>
+      <c r="G144" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="0">
+        <v>51057</v>
+      </c>
+      <c r="B145" s="0">
+        <v>0</v>
+      </c>
+      <c r="C145" s="0">
+        <v>0</v>
+      </c>
+      <c r="D145" s="0">
+        <v>0</v>
+      </c>
+      <c r="E145" s="0">
+        <v>0</v>
+      </c>
+      <c r="F145" s="0">
+        <v>0</v>
+      </c>
+      <c r="G145" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="0">
+        <v>52768</v>
+      </c>
+      <c r="B146" s="0">
+        <v>0</v>
+      </c>
+      <c r="C146" s="0">
+        <v>0</v>
+      </c>
+      <c r="D146" s="0">
+        <v>0</v>
+      </c>
+      <c r="E146" s="0">
+        <v>0</v>
+      </c>
+      <c r="F146" s="0">
+        <v>0</v>
+      </c>
+      <c r="G146" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="0">
+        <v>54804</v>
+      </c>
+      <c r="B147" s="0">
+        <v>4</v>
+      </c>
+      <c r="C147" s="0">
+        <v>3</v>
+      </c>
+      <c r="D147" s="0">
+        <v>0.87</v>
+      </c>
+      <c r="E147" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F147" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G147" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="0">
+        <v>46278</v>
+      </c>
+      <c r="B148" s="0">
+        <v>0</v>
+      </c>
+      <c r="C148" s="0">
+        <v>0</v>
+      </c>
+      <c r="D148" s="0">
+        <v>0</v>
+      </c>
+      <c r="E148" s="0">
+        <v>0</v>
+      </c>
+      <c r="F148" s="0">
+        <v>0</v>
+      </c>
+      <c r="G148" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="0">
+        <v>17295</v>
+      </c>
+      <c r="B149" s="0">
+        <v>0</v>
+      </c>
+      <c r="C149" s="0">
+        <v>0</v>
+      </c>
+      <c r="D149" s="0">
+        <v>0</v>
+      </c>
+      <c r="E149" s="0">
+        <v>0</v>
+      </c>
+      <c r="F149" s="0">
+        <v>0</v>
+      </c>
+      <c r="G149" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="0">
+        <v>55097</v>
+      </c>
+      <c r="B150" s="0">
+        <v>0</v>
+      </c>
+      <c r="C150" s="0">
+        <v>0</v>
+      </c>
+      <c r="D150" s="0">
+        <v>0</v>
+      </c>
+      <c r="E150" s="0">
+        <v>0</v>
+      </c>
+      <c r="F150" s="0">
+        <v>0</v>
+      </c>
+      <c r="G150" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="0">
+        <v>55030</v>
+      </c>
+      <c r="B151" s="0">
+        <v>0</v>
+      </c>
+      <c r="C151" s="0">
+        <v>0</v>
+      </c>
+      <c r="D151" s="0">
+        <v>0</v>
+      </c>
+      <c r="E151" s="0">
+        <v>0</v>
+      </c>
+      <c r="F151" s="0">
+        <v>0</v>
+      </c>
+      <c r="G151" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="0">
+        <v>44407</v>
+      </c>
+      <c r="B152" s="0">
+        <v>0</v>
+      </c>
+      <c r="C152" s="0">
+        <v>0</v>
+      </c>
+      <c r="D152" s="0">
+        <v>0</v>
+      </c>
+      <c r="E152" s="0">
+        <v>0</v>
+      </c>
+      <c r="F152" s="0">
+        <v>0</v>
+      </c>
+      <c r="G152" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="0">
+        <v>55040</v>
+      </c>
+      <c r="B153" s="0">
+        <v>0</v>
+      </c>
+      <c r="C153" s="0">
+        <v>0</v>
+      </c>
+      <c r="D153" s="0">
+        <v>0</v>
+      </c>
+      <c r="E153" s="0">
+        <v>0</v>
+      </c>
+      <c r="F153" s="0">
+        <v>0</v>
+      </c>
+      <c r="G153" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="0">
+        <v>48903</v>
+      </c>
+      <c r="B154" s="0">
+        <v>0</v>
+      </c>
+      <c r="C154" s="0">
+        <v>0</v>
+      </c>
+      <c r="D154" s="0">
+        <v>0</v>
+      </c>
+      <c r="E154" s="0">
+        <v>0</v>
+      </c>
+      <c r="F154" s="0">
+        <v>0</v>
+      </c>
+      <c r="G154" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="0">
+        <v>44876</v>
+      </c>
+      <c r="B155" s="0">
+        <v>0</v>
+      </c>
+      <c r="C155" s="0">
+        <v>0</v>
+      </c>
+      <c r="D155" s="0">
+        <v>0</v>
+      </c>
+      <c r="E155" s="0">
+        <v>0</v>
+      </c>
+      <c r="F155" s="0">
+        <v>0</v>
+      </c>
+      <c r="G155" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="0">
+        <v>43100</v>
+      </c>
+      <c r="B156" s="0">
+        <v>3</v>
+      </c>
+      <c r="C156" s="0">
+        <v>1</v>
+      </c>
+      <c r="D156" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E156" s="0">
+        <v>4</v>
+      </c>
+      <c r="F156" s="0">
+        <v>200</v>
+      </c>
+      <c r="G156" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="0">
+        <v>46286</v>
+      </c>
+      <c r="B157" s="0">
+        <v>0</v>
+      </c>
+      <c r="C157" s="0">
+        <v>0</v>
+      </c>
+      <c r="D157" s="0">
+        <v>0</v>
+      </c>
+      <c r="E157" s="0">
+        <v>0</v>
+      </c>
+      <c r="F157" s="0">
+        <v>0</v>
+      </c>
+      <c r="G157" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="0">
+        <v>47448</v>
+      </c>
+      <c r="B158" s="0">
+        <v>0</v>
+      </c>
+      <c r="C158" s="0">
+        <v>0</v>
+      </c>
+      <c r="D158" s="0">
+        <v>0</v>
+      </c>
+      <c r="E158" s="0">
+        <v>0</v>
+      </c>
+      <c r="F158" s="0">
+        <v>0</v>
+      </c>
+      <c r="G158" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="0">
+        <v>46570</v>
+      </c>
+      <c r="B159" s="0">
+        <v>4</v>
+      </c>
+      <c r="C159" s="0">
+        <v>3</v>
+      </c>
+      <c r="D159" s="0">
+        <v>0.5</v>
+      </c>
+      <c r="E159" s="0">
+        <v>6219</v>
+      </c>
+      <c r="F159" s="0">
+        <v>0.80000000000000004</v>
+      </c>
+      <c r="G159" s="0">
         <v>1</v>
       </c>
     </row>

</xml_diff>